<commit_message>
fine progettazione e creazione progetto con inizio sprint 1
</commit_message>
<xml_diff>
--- a/7_Allegati/Sprint-planning.xlsx
+++ b/7_Allegati/Sprint-planning.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ckw924\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nqy271\BrutalBumperCars\bianchi-ciaponi-brutal-bumper-cars\7_Allegati\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00CD6B61-D1B5-41E2-B980-11C1693EC3E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A62B3FC3-F495-46FA-90D6-D1FA897E5FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gantt Orario Dettagliato" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="215">
   <si>
     <t>Sprint</t>
   </si>
@@ -783,6 +783,30 @@
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="14">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF5B9BD5"/>
+          <bgColor rgb="FF5B9BD5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF5B9BD5"/>
+          <bgColor rgb="FF5B9BD5"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -924,30 +948,6 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFED7D31"/>
           <bgColor rgb="FFED7D31"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF5B9BD5"/>
-          <bgColor rgb="FF5B9BD5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF5B9BD5"/>
-          <bgColor rgb="FF5B9BD5"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2012,11 +2012,11 @@
         <v>4</v>
       </c>
       <c r="F3" s="3">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G3" s="5">
-        <f t="shared" ref="F3:G12" si="0">COUNTIF(H3:FS3, "X")</f>
-        <v>12</v>
+        <f t="shared" ref="G3:G12" si="0">COUNTIF(H3:FS3, "X")</f>
+        <v>11</v>
       </c>
       <c r="H3" s="6"/>
       <c r="I3" s="6"/>
@@ -2059,9 +2059,7 @@
       <c r="Z3" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="AA3" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
       <c r="AD3" s="6"/>
@@ -2205,7 +2203,6 @@
       <c r="FL3" s="6"/>
       <c r="FM3" s="6"/>
       <c r="FN3" s="6"/>
-      <c r="FO3" s="6"/>
     </row>
     <row r="4" spans="1:175" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
@@ -2249,7 +2246,9 @@
       <c r="X4" s="6"/>
       <c r="Y4" s="6"/>
       <c r="Z4" s="6"/>
-      <c r="AA4" s="6"/>
+      <c r="AA4" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="AB4" s="3" t="s">
         <v>179</v>
       </c>
@@ -2283,9 +2282,7 @@
       <c r="AL4" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="AM4" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="AM4" s="6"/>
       <c r="AN4" s="6"/>
       <c r="AO4" s="6"/>
       <c r="AP4" s="6"/>
@@ -2417,7 +2414,6 @@
       <c r="FL4" s="6"/>
       <c r="FM4" s="6"/>
       <c r="FN4" s="6"/>
-      <c r="FO4" s="6"/>
     </row>
     <row r="5" spans="1:175" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
@@ -2473,7 +2469,9 @@
       <c r="AJ5" s="6"/>
       <c r="AK5" s="6"/>
       <c r="AL5" s="6"/>
-      <c r="AM5" s="6"/>
+      <c r="AM5" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="AN5" s="3" t="s">
         <v>179</v>
       </c>
@@ -2483,9 +2481,7 @@
       <c r="AP5" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="AQ5" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="AQ5" s="6"/>
       <c r="AR5" s="6"/>
       <c r="AS5" s="6"/>
       <c r="AT5" s="6"/>
@@ -2613,7 +2609,6 @@
       <c r="FL5" s="6"/>
       <c r="FM5" s="6"/>
       <c r="FN5" s="6"/>
-      <c r="FO5" s="6"/>
     </row>
     <row r="6" spans="1:175" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
@@ -2673,7 +2668,9 @@
       <c r="AN6" s="6"/>
       <c r="AO6" s="6"/>
       <c r="AP6" s="6"/>
-      <c r="AQ6" s="6"/>
+      <c r="AQ6" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="AR6" s="3" t="s">
         <v>179</v>
       </c>
@@ -2695,9 +2692,7 @@
       <c r="AX6" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="AY6" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="AY6" s="6"/>
       <c r="AZ6" s="6"/>
       <c r="BA6" s="6"/>
       <c r="BB6" s="6"/>
@@ -2817,7 +2812,6 @@
       <c r="FL6" s="6"/>
       <c r="FM6" s="6"/>
       <c r="FN6" s="6"/>
-      <c r="FO6" s="6"/>
     </row>
     <row r="7" spans="1:175" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
@@ -2885,7 +2879,9 @@
       <c r="AV7" s="6"/>
       <c r="AW7" s="6"/>
       <c r="AX7" s="6"/>
-      <c r="AY7" s="6"/>
+      <c r="AY7" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="AZ7" s="3" t="s">
         <v>179</v>
       </c>
@@ -2955,9 +2951,7 @@
       <c r="BV7" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="BW7" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="BW7" s="6"/>
       <c r="BX7" s="6"/>
       <c r="BY7" s="6"/>
       <c r="BZ7" s="6"/>
@@ -3053,7 +3047,6 @@
       <c r="FL7" s="6"/>
       <c r="FM7" s="6"/>
       <c r="FN7" s="6"/>
-      <c r="FO7" s="6"/>
     </row>
     <row r="8" spans="1:175" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
@@ -3145,7 +3138,9 @@
       <c r="BT8" s="6"/>
       <c r="BU8" s="6"/>
       <c r="BV8" s="6"/>
-      <c r="BW8" s="6"/>
+      <c r="BW8" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="BX8" s="3" t="s">
         <v>179</v>
       </c>
@@ -3215,9 +3210,7 @@
       <c r="CT8" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="CU8" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="CU8" s="6"/>
       <c r="CV8" s="6"/>
       <c r="CW8" s="6"/>
       <c r="CX8" s="6"/>
@@ -3289,7 +3282,6 @@
       <c r="FL8" s="6"/>
       <c r="FM8" s="6"/>
       <c r="FN8" s="6"/>
-      <c r="FO8" s="6"/>
     </row>
     <row r="9" spans="1:175" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
@@ -3405,7 +3397,9 @@
       <c r="CR9" s="6"/>
       <c r="CS9" s="6"/>
       <c r="CT9" s="6"/>
-      <c r="CU9" s="6"/>
+      <c r="CU9" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="CV9" s="3" t="s">
         <v>179</v>
       </c>
@@ -3475,9 +3469,7 @@
       <c r="DR9" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="DS9" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="DS9" s="6"/>
       <c r="DT9" s="6"/>
       <c r="DU9" s="6"/>
       <c r="DV9" s="6"/>
@@ -3525,7 +3517,6 @@
       <c r="FL9" s="6"/>
       <c r="FM9" s="6"/>
       <c r="FN9" s="6"/>
-      <c r="FO9" s="6"/>
     </row>
     <row r="10" spans="1:175" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
@@ -3665,7 +3656,9 @@
       <c r="DP10" s="6"/>
       <c r="DQ10" s="6"/>
       <c r="DR10" s="6"/>
-      <c r="DS10" s="6"/>
+      <c r="DS10" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="DT10" s="3" t="s">
         <v>179</v>
       </c>
@@ -3711,9 +3704,7 @@
       <c r="EH10" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="EI10" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="EI10" s="6"/>
       <c r="EJ10" s="6"/>
       <c r="EK10" s="6"/>
       <c r="EL10" s="6"/>
@@ -3745,7 +3736,6 @@
       <c r="FL10" s="6"/>
       <c r="FM10" s="6"/>
       <c r="FN10" s="6"/>
-      <c r="FO10" s="6"/>
     </row>
     <row r="11" spans="1:175" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
@@ -3901,7 +3891,9 @@
       <c r="EF11" s="6"/>
       <c r="EG11" s="6"/>
       <c r="EH11" s="6"/>
-      <c r="EI11" s="6"/>
+      <c r="EI11" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="EJ11" s="3" t="s">
         <v>179</v>
       </c>
@@ -3923,9 +3915,7 @@
       <c r="EP11" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="EQ11" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="EQ11" s="6"/>
       <c r="ER11" s="6"/>
       <c r="ES11" s="6"/>
       <c r="ET11" s="6"/>
@@ -3949,7 +3939,6 @@
       <c r="FL11" s="6"/>
       <c r="FM11" s="6"/>
       <c r="FN11" s="6"/>
-      <c r="FO11" s="6"/>
     </row>
     <row r="12" spans="1:175" ht="60" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
@@ -4113,7 +4102,9 @@
       <c r="EN12" s="6"/>
       <c r="EO12" s="6"/>
       <c r="EP12" s="6"/>
-      <c r="EQ12" s="6"/>
+      <c r="EQ12" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="ER12" s="3" t="s">
         <v>179</v>
       </c>
@@ -4181,66 +4172,63 @@
         <v>179</v>
       </c>
       <c r="FN12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FO12" s="3" t="s">
         <v>179</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:FS2 H3:FO3">
-    <cfRule type="cellIs" dxfId="13" priority="1" operator="equal">
+  <conditionalFormatting sqref="H4:FN6">
+    <cfRule type="cellIs" dxfId="13" priority="5" operator="equal">
       <formula>"X"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="6" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H4:FO6">
-    <cfRule type="cellIs" dxfId="11" priority="5" operator="equal">
+  <conditionalFormatting sqref="H7:FN7">
+    <cfRule type="cellIs" dxfId="11" priority="11" operator="equal">
       <formula>"X"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="12" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H7:FO7">
-    <cfRule type="cellIs" dxfId="9" priority="11" operator="equal">
+  <conditionalFormatting sqref="H8:FN8">
+    <cfRule type="cellIs" dxfId="9" priority="13" operator="equal">
       <formula>"X"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="14" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H8:FO8">
-    <cfRule type="cellIs" dxfId="7" priority="13" operator="equal">
+  <conditionalFormatting sqref="H9:FN9">
+    <cfRule type="cellIs" dxfId="7" priority="15" operator="equal">
       <formula>"X"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="16" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H9:FO9">
-    <cfRule type="cellIs" dxfId="5" priority="15" operator="equal">
+  <conditionalFormatting sqref="H10:FN11">
+    <cfRule type="cellIs" dxfId="5" priority="17" operator="equal">
       <formula>"X"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="18" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H10:FO11">
-    <cfRule type="cellIs" dxfId="3" priority="17" operator="equal">
+  <conditionalFormatting sqref="H12:FN12">
+    <cfRule type="cellIs" dxfId="3" priority="21" operator="equal">
       <formula>"X"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="22" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H12:FO12">
-    <cfRule type="cellIs" dxfId="1" priority="21" operator="equal">
+  <conditionalFormatting sqref="H2:FS2 H3:FN3">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"X"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Sprint 1 Review Update
</commit_message>
<xml_diff>
--- a/7_Allegati/Sprint-planning.xlsx
+++ b/7_Allegati/Sprint-planning.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nqy271\BrutalBumperCars\bianchi-ciaponi-brutal-bumper-cars\7_Allegati\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Scuola\Anno_4\BrutalBumperCars(BBC)\7_Allegati\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A62B3FC3-F495-46FA-90D6-D1FA897E5FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{272B6EFA-EEE0-4F3E-8106-833AA463CE23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gantt Orario Dettagliato" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="216">
   <si>
     <t>Sprint</t>
   </si>
@@ -583,10 +583,6 @@
   </si>
   <si>
     <t>Accesso e modifica delle impostazioni di gioco.</t>
-  </si>
-  <si>
-    <t>• Dal menu principale voglio poter aprire le impostazioni di gioco.
-• Dalle impostazioni voglio poter cambiare le impostazioni.</t>
   </si>
   <si>
     <t>Sprint 2</t>
@@ -693,13 +689,20 @@
   <si>
     <t>• Tramite l'apposito comando (SHIFT) posso driftare.
 • Posso manovrare la macchina durante il drift.</t>
+  </si>
+  <si>
+    <t>• Voglio poter aprire le impostazioni di gioco.
+• Dalle impostazioni voglio poter cambiare le impostazioni.</t>
+  </si>
+  <si>
+    <t>169</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -717,6 +720,12 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -782,7 +791,103 @@
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="14">
+  <dxfs count="22">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFED7D31"/>
+          <bgColor rgb="FFED7D31"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFED7D31"/>
+          <bgColor rgb="FFED7D31"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFED7D31"/>
+          <bgColor rgb="FFED7D31"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFED7D31"/>
+          <bgColor rgb="FFED7D31"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFED7D31"/>
+          <bgColor rgb="FFED7D31"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFED7D31"/>
+          <bgColor rgb="FFED7D31"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFED7D31"/>
+          <bgColor rgb="FFED7D31"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFED7D31"/>
+          <bgColor rgb="FFED7D31"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -1249,7 +1354,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:FS12"/>
+  <dimension ref="A1:FT13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="10" customWidth="1"/>
@@ -1257,10 +1362,10 @@
     <col min="4" max="4" width="40" customWidth="1"/>
     <col min="5" max="5" width="6" customWidth="1"/>
     <col min="6" max="7" width="12" customWidth="1"/>
-    <col min="8" max="175" width="2.42578125" customWidth="1"/>
+    <col min="8" max="176" width="2.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:175" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:176" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1786,8 +1891,11 @@
       <c r="FS1" s="2" t="s">
         <v>174</v>
       </c>
+      <c r="FT1" s="2" t="s">
+        <v>215</v>
+      </c>
     </row>
-    <row r="2" spans="1:175" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:176" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>175</v>
       </c>
@@ -1807,8 +1915,8 @@
         <v>8</v>
       </c>
       <c r="G2" s="5">
-        <f>COUNTIF(H2:FS2, "X")</f>
-        <v>8</v>
+        <f>COUNTIF(H2:FT2, "X")</f>
+        <v>14</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>179</v>
@@ -1834,12 +1942,24 @@
       <c r="O2" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="6"/>
-      <c r="S2" s="6"/>
-      <c r="T2" s="6"/>
-      <c r="U2" s="6"/>
+      <c r="P2" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="V2" s="6"/>
       <c r="W2" s="6"/>
       <c r="X2" s="6"/>
@@ -1994,8 +2114,9 @@
       <c r="FQ2" s="6"/>
       <c r="FR2" s="6"/>
       <c r="FS2" s="6"/>
+      <c r="FT2" s="6"/>
     </row>
-    <row r="3" spans="1:175" ht="60" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:176" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>175</v>
       </c>
@@ -2006,7 +2127,7 @@
         <v>181</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>182</v>
+        <v>214</v>
       </c>
       <c r="E3" s="3">
         <v>4</v>
@@ -2015,8 +2136,8 @@
         <v>11</v>
       </c>
       <c r="G3" s="5">
-        <f t="shared" ref="G3:G12" si="0">COUNTIF(H3:FS3, "X")</f>
-        <v>11</v>
+        <f t="shared" ref="G3:G13" si="0">COUNTIF(H3:FT3, "X")</f>
+        <v>10</v>
       </c>
       <c r="H3" s="6"/>
       <c r="I3" s="6"/>
@@ -2044,12 +2165,8 @@
       <c r="U3" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="V3" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="W3" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="V3" s="3"/>
+      <c r="W3" s="3"/>
       <c r="X3" s="3" t="s">
         <v>179</v>
       </c>
@@ -2059,7 +2176,9 @@
       <c r="Z3" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="AA3" s="6"/>
+      <c r="AA3" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="AB3" s="6"/>
       <c r="AC3" s="6"/>
       <c r="AD3" s="6"/>
@@ -2203,29 +2322,30 @@
       <c r="FL3" s="6"/>
       <c r="FM3" s="6"/>
       <c r="FN3" s="6"/>
+      <c r="FO3" s="6"/>
     </row>
-    <row r="4" spans="1:175" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:176" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>186</v>
+        <v>214</v>
       </c>
       <c r="E4" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F4" s="3">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="G4" s="5">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="H4" s="6"/>
       <c r="I4" s="6"/>
@@ -2235,20 +2355,18 @@
       <c r="M4" s="6"/>
       <c r="N4" s="6"/>
       <c r="O4" s="6"/>
-      <c r="P4" s="6"/>
-      <c r="Q4" s="6"/>
-      <c r="R4" s="6"/>
-      <c r="S4" s="6"/>
-      <c r="T4" s="6"/>
-      <c r="U4" s="6"/>
-      <c r="V4" s="6"/>
-      <c r="W4" s="6"/>
-      <c r="X4" s="6"/>
-      <c r="Y4" s="6"/>
-      <c r="Z4" s="6"/>
-      <c r="AA4" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="U4" s="3"/>
+      <c r="V4" s="3"/>
+      <c r="W4" s="3"/>
+      <c r="X4" s="3"/>
+      <c r="Y4" s="3"/>
+      <c r="Z4" s="3"/>
+      <c r="AA4" s="3"/>
       <c r="AB4" s="3" t="s">
         <v>179</v>
       </c>
@@ -2261,27 +2379,13 @@
       <c r="AE4" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="AF4" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AG4" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AH4" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AI4" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AJ4" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AK4" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AL4" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="AF4" s="6"/>
+      <c r="AG4" s="6"/>
+      <c r="AH4" s="6"/>
+      <c r="AI4" s="6"/>
+      <c r="AJ4" s="6"/>
+      <c r="AK4" s="6"/>
+      <c r="AL4" s="6"/>
       <c r="AM4" s="6"/>
       <c r="AN4" s="6"/>
       <c r="AO4" s="6"/>
@@ -2414,29 +2518,30 @@
       <c r="FL4" s="6"/>
       <c r="FM4" s="6"/>
       <c r="FN4" s="6"/>
+      <c r="FO4" s="6"/>
     </row>
-    <row r="5" spans="1:175" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:176" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>187</v>
-      </c>
       <c r="C5" s="4" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="E5" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F5" s="3">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G5" s="5">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="H5" s="6"/>
       <c r="I5" s="6"/>
@@ -2458,29 +2563,45 @@
       <c r="Y5" s="6"/>
       <c r="Z5" s="6"/>
       <c r="AA5" s="6"/>
-      <c r="AB5" s="6"/>
-      <c r="AC5" s="6"/>
-      <c r="AD5" s="6"/>
-      <c r="AE5" s="6"/>
-      <c r="AF5" s="6"/>
-      <c r="AG5" s="6"/>
-      <c r="AH5" s="6"/>
-      <c r="AI5" s="6"/>
-      <c r="AJ5" s="6"/>
-      <c r="AK5" s="6"/>
-      <c r="AL5" s="6"/>
+      <c r="AB5" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AC5" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AD5" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AE5" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AF5" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AG5" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AH5" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AI5" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ5" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AK5" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AL5" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="AM5" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="AN5" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AO5" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AP5" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="AN5" s="6"/>
+      <c r="AO5" s="6"/>
+      <c r="AP5" s="6"/>
       <c r="AQ5" s="6"/>
       <c r="AR5" s="6"/>
       <c r="AS5" s="6"/>
@@ -2609,29 +2730,30 @@
       <c r="FL5" s="6"/>
       <c r="FM5" s="6"/>
       <c r="FN5" s="6"/>
+      <c r="FO5" s="6"/>
     </row>
-    <row r="6" spans="1:175" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:176" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="E6" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6" s="3">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G6" s="5">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H6" s="6"/>
       <c r="I6" s="6"/>
@@ -2665,33 +2787,25 @@
       <c r="AK6" s="6"/>
       <c r="AL6" s="6"/>
       <c r="AM6" s="6"/>
-      <c r="AN6" s="6"/>
-      <c r="AO6" s="6"/>
-      <c r="AP6" s="6"/>
+      <c r="AN6" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AO6" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AP6" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="AQ6" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="AR6" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AS6" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AT6" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AU6" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AV6" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AW6" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AX6" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="AR6" s="6"/>
+      <c r="AS6" s="6"/>
+      <c r="AT6" s="6"/>
+      <c r="AU6" s="6"/>
+      <c r="AV6" s="6"/>
+      <c r="AW6" s="6"/>
+      <c r="AX6" s="6"/>
       <c r="AY6" s="6"/>
       <c r="AZ6" s="6"/>
       <c r="BA6" s="6"/>
@@ -2812,29 +2926,30 @@
       <c r="FL6" s="6"/>
       <c r="FM6" s="6"/>
       <c r="FN6" s="6"/>
+      <c r="FO6" s="6"/>
     </row>
-    <row r="7" spans="1:175" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:176" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="E7" s="3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F7" s="3">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="G7" s="5">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="H7" s="6"/>
       <c r="I7" s="6"/>
@@ -2872,85 +2987,53 @@
       <c r="AO7" s="6"/>
       <c r="AP7" s="6"/>
       <c r="AQ7" s="6"/>
-      <c r="AR7" s="6"/>
-      <c r="AS7" s="6"/>
-      <c r="AT7" s="6"/>
-      <c r="AU7" s="6"/>
-      <c r="AV7" s="6"/>
-      <c r="AW7" s="6"/>
-      <c r="AX7" s="6"/>
+      <c r="AR7" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AS7" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AT7" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AU7" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AV7" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AW7" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AX7" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="AY7" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="AZ7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BA7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BB7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BC7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BD7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BE7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BF7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BG7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BH7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BI7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BJ7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BK7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BL7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BM7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BN7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BO7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BP7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BQ7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BR7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BS7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BT7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BU7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BV7" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="AZ7" s="6"/>
+      <c r="BA7" s="6"/>
+      <c r="BB7" s="6"/>
+      <c r="BC7" s="6"/>
+      <c r="BD7" s="6"/>
+      <c r="BE7" s="6"/>
+      <c r="BF7" s="6"/>
+      <c r="BG7" s="6"/>
+      <c r="BH7" s="6"/>
+      <c r="BI7" s="6"/>
+      <c r="BJ7" s="6"/>
+      <c r="BK7" s="6"/>
+      <c r="BL7" s="6"/>
+      <c r="BM7" s="6"/>
+      <c r="BN7" s="6"/>
+      <c r="BO7" s="6"/>
+      <c r="BP7" s="6"/>
+      <c r="BQ7" s="6"/>
+      <c r="BR7" s="6"/>
+      <c r="BS7" s="6"/>
+      <c r="BT7" s="6"/>
+      <c r="BU7" s="6"/>
+      <c r="BV7" s="6"/>
       <c r="BW7" s="6"/>
       <c r="BX7" s="6"/>
       <c r="BY7" s="6"/>
@@ -3047,22 +3130,23 @@
       <c r="FL7" s="6"/>
       <c r="FM7" s="6"/>
       <c r="FN7" s="6"/>
+      <c r="FO7" s="6"/>
     </row>
-    <row r="8" spans="1:175" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:176" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E8" s="3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F8" s="3">
         <v>24</v>
@@ -3115,101 +3199,101 @@
       <c r="AW8" s="6"/>
       <c r="AX8" s="6"/>
       <c r="AY8" s="6"/>
-      <c r="AZ8" s="6"/>
-      <c r="BA8" s="6"/>
-      <c r="BB8" s="6"/>
-      <c r="BC8" s="6"/>
-      <c r="BD8" s="6"/>
-      <c r="BE8" s="6"/>
-      <c r="BF8" s="6"/>
-      <c r="BG8" s="6"/>
-      <c r="BH8" s="6"/>
-      <c r="BI8" s="6"/>
-      <c r="BJ8" s="6"/>
-      <c r="BK8" s="6"/>
-      <c r="BL8" s="6"/>
-      <c r="BM8" s="6"/>
-      <c r="BN8" s="6"/>
-      <c r="BO8" s="6"/>
-      <c r="BP8" s="6"/>
-      <c r="BQ8" s="6"/>
-      <c r="BR8" s="6"/>
-      <c r="BS8" s="6"/>
-      <c r="BT8" s="6"/>
-      <c r="BU8" s="6"/>
-      <c r="BV8" s="6"/>
+      <c r="AZ8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BA8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BB8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BC8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BD8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BE8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BF8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BG8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BH8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BI8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BJ8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BK8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BL8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BM8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BN8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BO8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BP8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BQ8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BR8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BS8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BT8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BU8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BV8" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="BW8" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="BX8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BY8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BZ8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CA8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CB8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CC8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CD8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CE8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CF8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CG8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CH8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CI8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CJ8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CK8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CL8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CM8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CN8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CO8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CP8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CQ8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CR8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CS8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CT8" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="BX8" s="6"/>
+      <c r="BY8" s="6"/>
+      <c r="BZ8" s="6"/>
+      <c r="CA8" s="6"/>
+      <c r="CB8" s="6"/>
+      <c r="CC8" s="6"/>
+      <c r="CD8" s="6"/>
+      <c r="CE8" s="6"/>
+      <c r="CF8" s="6"/>
+      <c r="CG8" s="6"/>
+      <c r="CH8" s="6"/>
+      <c r="CI8" s="6"/>
+      <c r="CJ8" s="6"/>
+      <c r="CK8" s="6"/>
+      <c r="CL8" s="6"/>
+      <c r="CM8" s="6"/>
+      <c r="CN8" s="6"/>
+      <c r="CO8" s="6"/>
+      <c r="CP8" s="6"/>
+      <c r="CQ8" s="6"/>
+      <c r="CR8" s="6"/>
+      <c r="CS8" s="6"/>
+      <c r="CT8" s="6"/>
       <c r="CU8" s="6"/>
       <c r="CV8" s="6"/>
       <c r="CW8" s="6"/>
@@ -3282,22 +3366,23 @@
       <c r="FL8" s="6"/>
       <c r="FM8" s="6"/>
       <c r="FN8" s="6"/>
+      <c r="FO8" s="6"/>
     </row>
-    <row r="9" spans="1:175" ht="90" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:176" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="E9" s="3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F9" s="3">
         <v>24</v>
@@ -3374,101 +3459,101 @@
       <c r="BU9" s="6"/>
       <c r="BV9" s="6"/>
       <c r="BW9" s="6"/>
-      <c r="BX9" s="6"/>
-      <c r="BY9" s="6"/>
-      <c r="BZ9" s="6"/>
-      <c r="CA9" s="6"/>
-      <c r="CB9" s="6"/>
-      <c r="CC9" s="6"/>
-      <c r="CD9" s="6"/>
-      <c r="CE9" s="6"/>
-      <c r="CF9" s="6"/>
-      <c r="CG9" s="6"/>
-      <c r="CH9" s="6"/>
-      <c r="CI9" s="6"/>
-      <c r="CJ9" s="6"/>
-      <c r="CK9" s="6"/>
-      <c r="CL9" s="6"/>
-      <c r="CM9" s="6"/>
-      <c r="CN9" s="6"/>
-      <c r="CO9" s="6"/>
-      <c r="CP9" s="6"/>
-      <c r="CQ9" s="6"/>
-      <c r="CR9" s="6"/>
-      <c r="CS9" s="6"/>
-      <c r="CT9" s="6"/>
+      <c r="BX9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BY9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BZ9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CA9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CB9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CC9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CD9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CE9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CF9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CG9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CH9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CI9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CJ9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CK9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CL9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CM9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CN9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CO9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CP9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CQ9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CR9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CS9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CT9" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="CU9" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="CV9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CW9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CX9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CY9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CZ9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DA9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DB9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DC9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DD9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DE9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DF9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DG9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DH9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DI9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DJ9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DK9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DL9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DM9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DN9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DO9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DP9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DQ9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DR9" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="CV9" s="6"/>
+      <c r="CW9" s="6"/>
+      <c r="CX9" s="6"/>
+      <c r="CY9" s="6"/>
+      <c r="CZ9" s="6"/>
+      <c r="DA9" s="6"/>
+      <c r="DB9" s="6"/>
+      <c r="DC9" s="6"/>
+      <c r="DD9" s="6"/>
+      <c r="DE9" s="6"/>
+      <c r="DF9" s="6"/>
+      <c r="DG9" s="6"/>
+      <c r="DH9" s="6"/>
+      <c r="DI9" s="6"/>
+      <c r="DJ9" s="6"/>
+      <c r="DK9" s="6"/>
+      <c r="DL9" s="6"/>
+      <c r="DM9" s="6"/>
+      <c r="DN9" s="6"/>
+      <c r="DO9" s="6"/>
+      <c r="DP9" s="6"/>
+      <c r="DQ9" s="6"/>
+      <c r="DR9" s="6"/>
       <c r="DS9" s="6"/>
       <c r="DT9" s="6"/>
       <c r="DU9" s="6"/>
@@ -3517,29 +3602,30 @@
       <c r="FL9" s="6"/>
       <c r="FM9" s="6"/>
       <c r="FN9" s="6"/>
+      <c r="FO9" s="6"/>
     </row>
-    <row r="10" spans="1:175" ht="45" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:176" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="E10" s="3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F10" s="3">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="G10" s="5">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="H10" s="6"/>
       <c r="I10" s="6"/>
@@ -3633,77 +3719,93 @@
       <c r="CS10" s="6"/>
       <c r="CT10" s="6"/>
       <c r="CU10" s="6"/>
-      <c r="CV10" s="6"/>
-      <c r="CW10" s="6"/>
-      <c r="CX10" s="6"/>
-      <c r="CY10" s="6"/>
-      <c r="CZ10" s="6"/>
-      <c r="DA10" s="6"/>
-      <c r="DB10" s="6"/>
-      <c r="DC10" s="6"/>
-      <c r="DD10" s="6"/>
-      <c r="DE10" s="6"/>
-      <c r="DF10" s="6"/>
-      <c r="DG10" s="6"/>
-      <c r="DH10" s="6"/>
-      <c r="DI10" s="6"/>
-      <c r="DJ10" s="6"/>
-      <c r="DK10" s="6"/>
-      <c r="DL10" s="6"/>
-      <c r="DM10" s="6"/>
-      <c r="DN10" s="6"/>
-      <c r="DO10" s="6"/>
-      <c r="DP10" s="6"/>
-      <c r="DQ10" s="6"/>
-      <c r="DR10" s="6"/>
+      <c r="CV10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CW10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CX10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CY10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CZ10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DA10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DB10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DC10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DD10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DE10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DF10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DG10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DH10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DI10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DJ10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DK10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DL10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DM10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DN10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DO10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DP10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DQ10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DR10" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="DS10" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="DT10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DU10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DV10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DW10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DX10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DY10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DZ10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EA10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EB10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EC10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="ED10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EE10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EF10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EG10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EH10" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="DT10" s="6"/>
+      <c r="DU10" s="6"/>
+      <c r="DV10" s="6"/>
+      <c r="DW10" s="6"/>
+      <c r="DX10" s="6"/>
+      <c r="DY10" s="6"/>
+      <c r="DZ10" s="6"/>
+      <c r="EA10" s="6"/>
+      <c r="EB10" s="6"/>
+      <c r="EC10" s="6"/>
+      <c r="ED10" s="6"/>
+      <c r="EE10" s="6"/>
+      <c r="EF10" s="6"/>
+      <c r="EG10" s="6"/>
+      <c r="EH10" s="6"/>
       <c r="EI10" s="6"/>
       <c r="EJ10" s="6"/>
       <c r="EK10" s="6"/>
@@ -3736,29 +3838,30 @@
       <c r="FL10" s="6"/>
       <c r="FM10" s="6"/>
       <c r="FN10" s="6"/>
+      <c r="FO10" s="6"/>
     </row>
-    <row r="11" spans="1:175" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:176" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>208</v>
-      </c>
       <c r="C11" s="4" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="E11" s="3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F11" s="3">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G11" s="5">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
@@ -3876,45 +3979,61 @@
       <c r="DQ11" s="6"/>
       <c r="DR11" s="6"/>
       <c r="DS11" s="6"/>
-      <c r="DT11" s="6"/>
-      <c r="DU11" s="6"/>
-      <c r="DV11" s="6"/>
-      <c r="DW11" s="6"/>
-      <c r="DX11" s="6"/>
-      <c r="DY11" s="6"/>
-      <c r="DZ11" s="6"/>
-      <c r="EA11" s="6"/>
-      <c r="EB11" s="6"/>
-      <c r="EC11" s="6"/>
-      <c r="ED11" s="6"/>
-      <c r="EE11" s="6"/>
-      <c r="EF11" s="6"/>
-      <c r="EG11" s="6"/>
-      <c r="EH11" s="6"/>
+      <c r="DT11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DU11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DV11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DW11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DX11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DY11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DZ11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EA11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EB11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EC11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="ED11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EE11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EF11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EG11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EH11" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="EI11" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="EJ11" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EK11" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EL11" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EM11" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EN11" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EO11" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EP11" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="EJ11" s="6"/>
+      <c r="EK11" s="6"/>
+      <c r="EL11" s="6"/>
+      <c r="EM11" s="6"/>
+      <c r="EN11" s="6"/>
+      <c r="EO11" s="6"/>
+      <c r="EP11" s="6"/>
       <c r="EQ11" s="6"/>
       <c r="ER11" s="6"/>
       <c r="ES11" s="6"/>
@@ -3939,29 +4058,30 @@
       <c r="FL11" s="6"/>
       <c r="FM11" s="6"/>
       <c r="FN11" s="6"/>
+      <c r="FO11" s="6"/>
     </row>
-    <row r="12" spans="1:175" ht="60" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:176" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="E12" s="3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F12" s="3">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="G12" s="5">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
@@ -4095,136 +4215,374 @@
       <c r="EG12" s="6"/>
       <c r="EH12" s="6"/>
       <c r="EI12" s="6"/>
-      <c r="EJ12" s="6"/>
-      <c r="EK12" s="6"/>
-      <c r="EL12" s="6"/>
-      <c r="EM12" s="6"/>
-      <c r="EN12" s="6"/>
-      <c r="EO12" s="6"/>
-      <c r="EP12" s="6"/>
+      <c r="EJ12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EK12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EL12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EM12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EN12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EO12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EP12" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="EQ12" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="ER12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="ES12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="ET12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EU12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EV12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EW12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EX12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EY12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EZ12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FA12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FB12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FC12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FD12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FE12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FF12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FG12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FH12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FI12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FJ12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FK12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FL12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FM12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FN12" s="3" t="s">
+      <c r="ER12" s="6"/>
+      <c r="ES12" s="6"/>
+      <c r="ET12" s="6"/>
+      <c r="EU12" s="6"/>
+      <c r="EV12" s="6"/>
+      <c r="EW12" s="6"/>
+      <c r="EX12" s="6"/>
+      <c r="EY12" s="6"/>
+      <c r="EZ12" s="6"/>
+      <c r="FA12" s="6"/>
+      <c r="FB12" s="6"/>
+      <c r="FC12" s="6"/>
+      <c r="FD12" s="6"/>
+      <c r="FE12" s="6"/>
+      <c r="FF12" s="6"/>
+      <c r="FG12" s="6"/>
+      <c r="FH12" s="6"/>
+      <c r="FI12" s="6"/>
+      <c r="FJ12" s="6"/>
+      <c r="FK12" s="6"/>
+      <c r="FL12" s="6"/>
+      <c r="FM12" s="6"/>
+      <c r="FN12" s="6"/>
+      <c r="FO12" s="6"/>
+    </row>
+    <row r="13" spans="1:176" ht="60" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="E13" s="3">
+        <v>5</v>
+      </c>
+      <c r="F13" s="3">
+        <v>24</v>
+      </c>
+      <c r="G13" s="5">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
+      <c r="N13" s="6"/>
+      <c r="O13" s="6"/>
+      <c r="P13" s="6"/>
+      <c r="Q13" s="6"/>
+      <c r="R13" s="6"/>
+      <c r="S13" s="6"/>
+      <c r="T13" s="6"/>
+      <c r="U13" s="6"/>
+      <c r="V13" s="6"/>
+      <c r="W13" s="6"/>
+      <c r="X13" s="6"/>
+      <c r="Y13" s="6"/>
+      <c r="Z13" s="6"/>
+      <c r="AA13" s="6"/>
+      <c r="AB13" s="6"/>
+      <c r="AC13" s="6"/>
+      <c r="AD13" s="6"/>
+      <c r="AE13" s="6"/>
+      <c r="AF13" s="6"/>
+      <c r="AG13" s="6"/>
+      <c r="AH13" s="6"/>
+      <c r="AI13" s="6"/>
+      <c r="AJ13" s="6"/>
+      <c r="AK13" s="6"/>
+      <c r="AL13" s="6"/>
+      <c r="AM13" s="6"/>
+      <c r="AN13" s="6"/>
+      <c r="AO13" s="6"/>
+      <c r="AP13" s="6"/>
+      <c r="AQ13" s="6"/>
+      <c r="AR13" s="6"/>
+      <c r="AS13" s="6"/>
+      <c r="AT13" s="6"/>
+      <c r="AU13" s="6"/>
+      <c r="AV13" s="6"/>
+      <c r="AW13" s="6"/>
+      <c r="AX13" s="6"/>
+      <c r="AY13" s="6"/>
+      <c r="AZ13" s="6"/>
+      <c r="BA13" s="6"/>
+      <c r="BB13" s="6"/>
+      <c r="BC13" s="6"/>
+      <c r="BD13" s="6"/>
+      <c r="BE13" s="6"/>
+      <c r="BF13" s="6"/>
+      <c r="BG13" s="6"/>
+      <c r="BH13" s="6"/>
+      <c r="BI13" s="6"/>
+      <c r="BJ13" s="6"/>
+      <c r="BK13" s="6"/>
+      <c r="BL13" s="6"/>
+      <c r="BM13" s="6"/>
+      <c r="BN13" s="6"/>
+      <c r="BO13" s="6"/>
+      <c r="BP13" s="6"/>
+      <c r="BQ13" s="6"/>
+      <c r="BR13" s="6"/>
+      <c r="BS13" s="6"/>
+      <c r="BT13" s="6"/>
+      <c r="BU13" s="6"/>
+      <c r="BV13" s="6"/>
+      <c r="BW13" s="6"/>
+      <c r="BX13" s="6"/>
+      <c r="BY13" s="6"/>
+      <c r="BZ13" s="6"/>
+      <c r="CA13" s="6"/>
+      <c r="CB13" s="6"/>
+      <c r="CC13" s="6"/>
+      <c r="CD13" s="6"/>
+      <c r="CE13" s="6"/>
+      <c r="CF13" s="6"/>
+      <c r="CG13" s="6"/>
+      <c r="CH13" s="6"/>
+      <c r="CI13" s="6"/>
+      <c r="CJ13" s="6"/>
+      <c r="CK13" s="6"/>
+      <c r="CL13" s="6"/>
+      <c r="CM13" s="6"/>
+      <c r="CN13" s="6"/>
+      <c r="CO13" s="6"/>
+      <c r="CP13" s="6"/>
+      <c r="CQ13" s="6"/>
+      <c r="CR13" s="6"/>
+      <c r="CS13" s="6"/>
+      <c r="CT13" s="6"/>
+      <c r="CU13" s="6"/>
+      <c r="CV13" s="6"/>
+      <c r="CW13" s="6"/>
+      <c r="CX13" s="6"/>
+      <c r="CY13" s="6"/>
+      <c r="CZ13" s="6"/>
+      <c r="DA13" s="6"/>
+      <c r="DB13" s="6"/>
+      <c r="DC13" s="6"/>
+      <c r="DD13" s="6"/>
+      <c r="DE13" s="6"/>
+      <c r="DF13" s="6"/>
+      <c r="DG13" s="6"/>
+      <c r="DH13" s="6"/>
+      <c r="DI13" s="6"/>
+      <c r="DJ13" s="6"/>
+      <c r="DK13" s="6"/>
+      <c r="DL13" s="6"/>
+      <c r="DM13" s="6"/>
+      <c r="DN13" s="6"/>
+      <c r="DO13" s="6"/>
+      <c r="DP13" s="6"/>
+      <c r="DQ13" s="6"/>
+      <c r="DR13" s="6"/>
+      <c r="DS13" s="6"/>
+      <c r="DT13" s="6"/>
+      <c r="DU13" s="6"/>
+      <c r="DV13" s="6"/>
+      <c r="DW13" s="6"/>
+      <c r="DX13" s="6"/>
+      <c r="DY13" s="6"/>
+      <c r="DZ13" s="6"/>
+      <c r="EA13" s="6"/>
+      <c r="EB13" s="6"/>
+      <c r="EC13" s="6"/>
+      <c r="ED13" s="6"/>
+      <c r="EE13" s="6"/>
+      <c r="EF13" s="6"/>
+      <c r="EG13" s="6"/>
+      <c r="EH13" s="6"/>
+      <c r="EI13" s="6"/>
+      <c r="EJ13" s="6"/>
+      <c r="EK13" s="6"/>
+      <c r="EL13" s="6"/>
+      <c r="EM13" s="6"/>
+      <c r="EN13" s="6"/>
+      <c r="EO13" s="6"/>
+      <c r="EP13" s="6"/>
+      <c r="EQ13" s="6"/>
+      <c r="ER13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="ES13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="ET13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EU13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EV13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EW13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EX13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EY13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EZ13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FA13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FB13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FC13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FD13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FE13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FF13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FG13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FH13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FI13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FJ13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FK13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FL13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FM13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FN13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FO13" s="3" t="s">
         <v>179</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H4:FN6">
-    <cfRule type="cellIs" dxfId="13" priority="5" operator="equal">
+  <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="H5:FO7">
+    <cfRule type="cellIs" dxfId="21" priority="13" operator="equal">
       <formula>"X"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="14" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H7:FN7">
-    <cfRule type="cellIs" dxfId="11" priority="11" operator="equal">
+  <conditionalFormatting sqref="H8:FO8">
+    <cfRule type="cellIs" dxfId="19" priority="19" operator="equal">
       <formula>"X"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="20" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H8:FN8">
-    <cfRule type="cellIs" dxfId="9" priority="13" operator="equal">
+  <conditionalFormatting sqref="H9:FO9">
+    <cfRule type="cellIs" dxfId="17" priority="21" operator="equal">
       <formula>"X"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="22" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H9:FN9">
-    <cfRule type="cellIs" dxfId="7" priority="15" operator="equal">
+  <conditionalFormatting sqref="H10:FO10">
+    <cfRule type="cellIs" dxfId="15" priority="23" operator="equal">
       <formula>"X"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="24" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H10:FN11">
-    <cfRule type="cellIs" dxfId="5" priority="17" operator="equal">
+  <conditionalFormatting sqref="H11:FO12">
+    <cfRule type="cellIs" dxfId="13" priority="25" operator="equal">
       <formula>"X"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="26" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H12:FN12">
-    <cfRule type="cellIs" dxfId="3" priority="21" operator="equal">
+  <conditionalFormatting sqref="H13:FO13">
+    <cfRule type="cellIs" dxfId="11" priority="29" operator="equal">
       <formula>"X"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="30" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:FS2 H3:FN3">
+  <conditionalFormatting sqref="H2:FT2 H3:FO3 H4:AA4 AF4:FO4">
+    <cfRule type="cellIs" dxfId="9" priority="9" operator="equal">
+      <formula>"X"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="8" priority="10" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AB4">
+    <cfRule type="cellIs" dxfId="7" priority="7" operator="equal">
+      <formula>"X"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="8" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AC4">
+    <cfRule type="cellIs" dxfId="5" priority="5" operator="equal">
+      <formula>"X"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="6" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD4">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+      <formula>"X"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AE4">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"X"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Progressi menu principale, con inizio sviluppo meccanica di spostamento tra pagine
</commit_message>
<xml_diff>
--- a/7_Allegati/Sprint-planning.xlsx
+++ b/7_Allegati/Sprint-planning.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Scuola\Anno_4\BrutalBumperCars(BBC)\7_Allegati\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{272B6EFA-EEE0-4F3E-8106-833AA463CE23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35162EE9-FEBD-4D01-B646-090F52C44F8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -791,79 +791,7 @@
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="22">
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFED7D31"/>
-          <bgColor rgb="FFED7D31"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFED7D31"/>
-          <bgColor rgb="FFED7D31"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFED7D31"/>
-          <bgColor rgb="FFED7D31"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFED7D31"/>
-          <bgColor rgb="FFED7D31"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFED7D31"/>
-          <bgColor rgb="FFED7D31"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFED7D31"/>
-          <bgColor rgb="FFED7D31"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="16">
     <dxf>
       <font>
         <b/>
@@ -2534,7 +2462,7 @@
         <v>185</v>
       </c>
       <c r="E5" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5" s="3">
         <v>12</v>
@@ -4503,86 +4431,62 @@
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <conditionalFormatting sqref="H5:FO7">
-    <cfRule type="cellIs" dxfId="21" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="13" operator="equal">
       <formula>"X"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="14" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H8:FO8">
-    <cfRule type="cellIs" dxfId="19" priority="19" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="19" operator="equal">
       <formula>"X"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="20" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H9:FO9">
-    <cfRule type="cellIs" dxfId="17" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="21" operator="equal">
       <formula>"X"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="22" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H10:FO10">
-    <cfRule type="cellIs" dxfId="15" priority="23" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="23" operator="equal">
       <formula>"X"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="24" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="24" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11:FO12">
-    <cfRule type="cellIs" dxfId="13" priority="25" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="25" operator="equal">
       <formula>"X"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="26" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="26" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H13:FO13">
-    <cfRule type="cellIs" dxfId="11" priority="29" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="29" operator="equal">
       <formula>"X"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="30" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="30" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:FT2 H3:FO3 H4:AA4 AF4:FO4">
-    <cfRule type="cellIs" dxfId="9" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="9" operator="equal">
       <formula>"X"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="10" operator="equal">
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AB4">
-    <cfRule type="cellIs" dxfId="7" priority="7" operator="equal">
-      <formula>"X"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="8" operator="equal">
-      <formula>"x"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AC4">
-    <cfRule type="cellIs" dxfId="5" priority="5" operator="equal">
-      <formula>"X"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="6" operator="equal">
-      <formula>"x"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AD4">
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
-      <formula>"X"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
-      <formula>"x"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AE4">
+  <conditionalFormatting sqref="AB4:AE4">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"X"</formula>
     </cfRule>

</xml_diff>

<commit_message>
aggiornamento sprint-planning e diario
</commit_message>
<xml_diff>
--- a/7_Allegati/Sprint-planning.xlsx
+++ b/7_Allegati/Sprint-planning.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Scuola\Anno_4\BrutalBumperCars(BBC)\7_Allegati\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nqy271\BrutalBumperCars\bianchi-ciaponi-brutal-bumper-cars\7_Allegati\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35162EE9-FEBD-4D01-B646-090F52C44F8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF412CC4-1571-4F60-85D0-5C8F8B3847DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gantt Orario Dettagliato" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="216">
   <si>
     <t>Sprint</t>
   </si>
@@ -2273,7 +2273,7 @@
       </c>
       <c r="G4" s="5">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H4" s="6"/>
       <c r="I4" s="6"/>
@@ -2307,8 +2307,12 @@
       <c r="AE4" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="AF4" s="6"/>
-      <c r="AG4" s="6"/>
+      <c r="AF4" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AG4" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="AH4" s="6"/>
       <c r="AI4" s="6"/>
       <c r="AJ4" s="6"/>
@@ -2469,7 +2473,7 @@
       </c>
       <c r="G5" s="5">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="H5" s="6"/>
       <c r="I5" s="6"/>
@@ -2500,33 +2504,15 @@
       <c r="AD5" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="AE5" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AF5" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AG5" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AH5" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AI5" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AJ5" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AK5" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AL5" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AM5" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="AE5" s="3"/>
+      <c r="AF5" s="3"/>
+      <c r="AG5" s="3"/>
+      <c r="AH5" s="3"/>
+      <c r="AI5" s="3"/>
+      <c r="AJ5" s="3"/>
+      <c r="AK5" s="3"/>
+      <c r="AL5" s="3"/>
+      <c r="AM5" s="3"/>
       <c r="AN5" s="6"/>
       <c r="AO5" s="6"/>
       <c r="AP5" s="6"/>
@@ -2681,7 +2667,7 @@
       </c>
       <c r="G6" s="5">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H6" s="6"/>
       <c r="I6" s="6"/>
@@ -2706,7 +2692,9 @@
       <c r="AB6" s="6"/>
       <c r="AC6" s="6"/>
       <c r="AD6" s="6"/>
-      <c r="AE6" s="6"/>
+      <c r="AE6" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="AF6" s="6"/>
       <c r="AG6" s="6"/>
       <c r="AH6" s="6"/>
@@ -2715,18 +2703,9 @@
       <c r="AK6" s="6"/>
       <c r="AL6" s="6"/>
       <c r="AM6" s="6"/>
-      <c r="AN6" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AO6" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AP6" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AQ6" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="AO6" s="3"/>
+      <c r="AP6" s="3"/>
+      <c r="AQ6" s="3"/>
       <c r="AR6" s="6"/>
       <c r="AS6" s="6"/>
       <c r="AT6" s="6"/>
@@ -2877,7 +2856,7 @@
       </c>
       <c r="G7" s="5">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="H7" s="6"/>
       <c r="I7" s="6"/>
@@ -2903,18 +2882,42 @@
       <c r="AC7" s="6"/>
       <c r="AD7" s="6"/>
       <c r="AE7" s="6"/>
-      <c r="AF7" s="6"/>
-      <c r="AG7" s="6"/>
-      <c r="AH7" s="6"/>
-      <c r="AI7" s="6"/>
-      <c r="AJ7" s="6"/>
-      <c r="AK7" s="6"/>
-      <c r="AL7" s="6"/>
-      <c r="AM7" s="6"/>
-      <c r="AN7" s="6"/>
-      <c r="AO7" s="6"/>
-      <c r="AP7" s="6"/>
-      <c r="AQ7" s="6"/>
+      <c r="AF7" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AG7" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AH7" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AI7" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ7" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AK7" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AL7" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AM7" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AN7" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AO7" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AP7" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AQ7" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="AR7" s="3" t="s">
         <v>179</v>
       </c>
@@ -4430,7 +4433,7 @@
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="H5:FO7">
+  <conditionalFormatting sqref="H5:FO5 AO6:FO6 H6:AM7 AN7:FO7">
     <cfRule type="cellIs" dxfId="15" priority="13" operator="equal">
       <formula>"X"</formula>
     </cfRule>
@@ -4478,7 +4481,7 @@
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:FT2 H3:FO3 H4:AA4 AF4:FO4">
+  <conditionalFormatting sqref="H2:FT2 H3:FO3 H4:AA4 AH4:FO4">
     <cfRule type="cellIs" dxfId="3" priority="9" operator="equal">
       <formula>"X"</formula>
     </cfRule>
@@ -4486,7 +4489,7 @@
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AB4:AE4">
+  <conditionalFormatting sqref="AB4:AG4">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"X"</formula>
     </cfRule>

</xml_diff>

<commit_message>
continuo creazione db, modifica sprint planning e diario
</commit_message>
<xml_diff>
--- a/7_Allegati/Sprint-planning.xlsx
+++ b/7_Allegati/Sprint-planning.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nqy271\BrutalBumperCars\bianchi-ciaponi-brutal-bumper-cars\7_Allegati\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF412CC4-1571-4F60-85D0-5C8F8B3847DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41D642B1-DB7F-4392-A01D-24B7166EC000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gantt Orario Dettagliato" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="216">
   <si>
     <t>Sprint</t>
   </si>
@@ -2856,7 +2856,7 @@
       </c>
       <c r="G7" s="5">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="H7" s="6"/>
       <c r="I7" s="6"/>
@@ -2894,54 +2894,26 @@
       <c r="AI7" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="AJ7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AK7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AL7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AM7" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="AJ7" s="3"/>
+      <c r="AK7" s="3"/>
+      <c r="AL7" s="3"/>
+      <c r="AM7" s="3"/>
       <c r="AN7" s="3" t="s">
         <v>179</v>
       </c>
       <c r="AO7" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="AP7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AQ7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AR7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AS7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AT7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AU7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AV7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AW7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AX7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="AY7" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="AP7" s="3"/>
+      <c r="AQ7" s="3"/>
+      <c r="AR7" s="3"/>
+      <c r="AS7" s="3"/>
+      <c r="AT7" s="3"/>
+      <c r="AU7" s="3"/>
+      <c r="AV7" s="3"/>
+      <c r="AW7" s="3"/>
+      <c r="AX7" s="3"/>
+      <c r="AY7" s="3"/>
       <c r="AZ7" s="6"/>
       <c r="BA7" s="6"/>
       <c r="BB7" s="6"/>

</xml_diff>

<commit_message>
modifica sprint planning, impostazione salvate su db (mancano i comandi) e diario
</commit_message>
<xml_diff>
--- a/7_Allegati/Sprint-planning.xlsx
+++ b/7_Allegati/Sprint-planning.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nqy271\BrutalBumperCars\bianchi-ciaponi-brutal-bumper-cars\7_Allegati\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41D642B1-DB7F-4392-A01D-24B7166EC000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D144A02-8816-4E75-BC35-6E0D98556A48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="217">
   <si>
     <t>Sprint</t>
   </si>
@@ -696,6 +696,9 @@
   </si>
   <si>
     <t>169</t>
+  </si>
+  <si>
+    <t>Extra</t>
   </si>
 </sst>
 </file>
@@ -1282,7 +1285,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:FT13"/>
+  <dimension ref="A1:FT14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="10" customWidth="1"/>
@@ -2064,7 +2067,7 @@
         <v>11</v>
       </c>
       <c r="G3" s="5">
-        <f t="shared" ref="G3:G13" si="0">COUNTIF(H3:FT3, "X")</f>
+        <f t="shared" ref="G3:G14" si="0">COUNTIF(H3:FT3, "X")</f>
         <v>10</v>
       </c>
       <c r="H3" s="6"/>
@@ -2855,7 +2858,7 @@
         <v>8</v>
       </c>
       <c r="G7" s="5">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="G7" si="1">COUNTIF(H7:FT7, "X")</f>
         <v>6</v>
       </c>
       <c r="H7" s="6"/>
@@ -3035,28 +3038,20 @@
       <c r="FN7" s="6"/>
       <c r="FO7" s="6"/>
     </row>
-    <row r="8" spans="1:176" ht="60" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:176" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>193</v>
-      </c>
+        <v>182</v>
+      </c>
+      <c r="B8" s="3"/>
       <c r="C8" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="E8" s="3">
-        <v>6</v>
-      </c>
-      <c r="F8" s="3">
-        <v>24</v>
-      </c>
+        <v>216</v>
+      </c>
+      <c r="D8" s="4"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
       <c r="G8" s="5">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="H8" s="6"/>
       <c r="I8" s="6"/>
@@ -3082,98 +3077,78 @@
       <c r="AC8" s="6"/>
       <c r="AD8" s="6"/>
       <c r="AE8" s="6"/>
-      <c r="AF8" s="6"/>
-      <c r="AG8" s="6"/>
-      <c r="AH8" s="6"/>
-      <c r="AI8" s="6"/>
-      <c r="AJ8" s="6"/>
-      <c r="AK8" s="6"/>
-      <c r="AL8" s="6"/>
-      <c r="AM8" s="6"/>
-      <c r="AN8" s="6"/>
-      <c r="AO8" s="6"/>
-      <c r="AP8" s="6"/>
-      <c r="AQ8" s="6"/>
-      <c r="AR8" s="6"/>
-      <c r="AS8" s="6"/>
-      <c r="AT8" s="6"/>
-      <c r="AU8" s="6"/>
-      <c r="AV8" s="6"/>
-      <c r="AW8" s="6"/>
-      <c r="AX8" s="6"/>
-      <c r="AY8" s="6"/>
-      <c r="AZ8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BA8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BB8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BC8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BD8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BE8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BF8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BG8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BH8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BI8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BJ8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BK8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BL8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BM8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BN8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BO8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BP8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BQ8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BR8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BS8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BT8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BU8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BV8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BW8" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="AF8" s="3"/>
+      <c r="AG8" s="3"/>
+      <c r="AH8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AI8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AJ8" s="3"/>
+      <c r="AK8" s="3"/>
+      <c r="AL8" s="3"/>
+      <c r="AM8" s="3"/>
+      <c r="AN8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AO8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AP8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AQ8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AR8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AS8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AT8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AU8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AV8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AW8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AX8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AY8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="AZ8" s="6"/>
+      <c r="BA8" s="6"/>
+      <c r="BB8" s="6"/>
+      <c r="BC8" s="6"/>
+      <c r="BD8" s="6"/>
+      <c r="BE8" s="6"/>
+      <c r="BF8" s="6"/>
+      <c r="BG8" s="6"/>
+      <c r="BH8" s="6"/>
+      <c r="BI8" s="6"/>
+      <c r="BJ8" s="6"/>
+      <c r="BK8" s="6"/>
+      <c r="BL8" s="6"/>
+      <c r="BM8" s="6"/>
+      <c r="BN8" s="6"/>
+      <c r="BO8" s="6"/>
+      <c r="BP8" s="6"/>
+      <c r="BQ8" s="6"/>
+      <c r="BR8" s="6"/>
+      <c r="BS8" s="6"/>
+      <c r="BT8" s="6"/>
+      <c r="BU8" s="6"/>
+      <c r="BV8" s="6"/>
+      <c r="BW8" s="6"/>
       <c r="BX8" s="6"/>
       <c r="BY8" s="6"/>
       <c r="BZ8" s="6"/>
@@ -3271,21 +3246,21 @@
       <c r="FN8" s="6"/>
       <c r="FO8" s="6"/>
     </row>
-    <row r="9" spans="1:176" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:176" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="E9" s="3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F9" s="3">
         <v>24</v>
@@ -3338,102 +3313,102 @@
       <c r="AW9" s="6"/>
       <c r="AX9" s="6"/>
       <c r="AY9" s="6"/>
-      <c r="AZ9" s="6"/>
-      <c r="BA9" s="6"/>
-      <c r="BB9" s="6"/>
-      <c r="BC9" s="6"/>
-      <c r="BD9" s="6"/>
-      <c r="BE9" s="6"/>
-      <c r="BF9" s="6"/>
-      <c r="BG9" s="6"/>
-      <c r="BH9" s="6"/>
-      <c r="BI9" s="6"/>
-      <c r="BJ9" s="6"/>
-      <c r="BK9" s="6"/>
-      <c r="BL9" s="6"/>
-      <c r="BM9" s="6"/>
-      <c r="BN9" s="6"/>
-      <c r="BO9" s="6"/>
-      <c r="BP9" s="6"/>
-      <c r="BQ9" s="6"/>
-      <c r="BR9" s="6"/>
-      <c r="BS9" s="6"/>
-      <c r="BT9" s="6"/>
-      <c r="BU9" s="6"/>
-      <c r="BV9" s="6"/>
-      <c r="BW9" s="6"/>
-      <c r="BX9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BY9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="BZ9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CA9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CB9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CC9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CD9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CE9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CF9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CG9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CH9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CI9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CJ9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CK9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CL9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CM9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CN9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CO9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CP9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CQ9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CR9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CS9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CT9" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CU9" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="AZ9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BA9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BB9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BC9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BD9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BE9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BF9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BG9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BH9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BI9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BJ9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BK9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BL9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BM9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BN9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BO9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BP9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BQ9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BR9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BS9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BT9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BU9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BV9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BW9" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BX9" s="6"/>
+      <c r="BY9" s="6"/>
+      <c r="BZ9" s="6"/>
+      <c r="CA9" s="6"/>
+      <c r="CB9" s="6"/>
+      <c r="CC9" s="6"/>
+      <c r="CD9" s="6"/>
+      <c r="CE9" s="6"/>
+      <c r="CF9" s="6"/>
+      <c r="CG9" s="6"/>
+      <c r="CH9" s="6"/>
+      <c r="CI9" s="6"/>
+      <c r="CJ9" s="6"/>
+      <c r="CK9" s="6"/>
+      <c r="CL9" s="6"/>
+      <c r="CM9" s="6"/>
+      <c r="CN9" s="6"/>
+      <c r="CO9" s="6"/>
+      <c r="CP9" s="6"/>
+      <c r="CQ9" s="6"/>
+      <c r="CR9" s="6"/>
+      <c r="CS9" s="6"/>
+      <c r="CT9" s="6"/>
+      <c r="CU9" s="6"/>
       <c r="CV9" s="6"/>
       <c r="CW9" s="6"/>
       <c r="CX9" s="6"/>
@@ -3507,21 +3482,21 @@
       <c r="FN9" s="6"/>
       <c r="FO9" s="6"/>
     </row>
-    <row r="10" spans="1:176" ht="90" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:176" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>202</v>
+        <v>191</v>
       </c>
       <c r="E10" s="3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F10" s="3">
         <v>24</v>
@@ -3598,102 +3573,102 @@
       <c r="BU10" s="6"/>
       <c r="BV10" s="6"/>
       <c r="BW10" s="6"/>
-      <c r="BX10" s="6"/>
-      <c r="BY10" s="6"/>
-      <c r="BZ10" s="6"/>
-      <c r="CA10" s="6"/>
-      <c r="CB10" s="6"/>
-      <c r="CC10" s="6"/>
-      <c r="CD10" s="6"/>
-      <c r="CE10" s="6"/>
-      <c r="CF10" s="6"/>
-      <c r="CG10" s="6"/>
-      <c r="CH10" s="6"/>
-      <c r="CI10" s="6"/>
-      <c r="CJ10" s="6"/>
-      <c r="CK10" s="6"/>
-      <c r="CL10" s="6"/>
-      <c r="CM10" s="6"/>
-      <c r="CN10" s="6"/>
-      <c r="CO10" s="6"/>
-      <c r="CP10" s="6"/>
-      <c r="CQ10" s="6"/>
-      <c r="CR10" s="6"/>
-      <c r="CS10" s="6"/>
-      <c r="CT10" s="6"/>
-      <c r="CU10" s="6"/>
-      <c r="CV10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CW10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CX10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CY10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="CZ10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DA10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DB10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DC10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DD10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DE10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DF10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DG10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DH10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DI10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DJ10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DK10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DL10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DM10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DN10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DO10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DP10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DQ10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DR10" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DS10" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="BX10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BY10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="BZ10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CA10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CB10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CC10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CD10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CE10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CF10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CG10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CH10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CI10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CJ10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CK10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CL10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CM10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CN10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CO10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CP10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CQ10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CR10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CS10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CT10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CU10" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CV10" s="6"/>
+      <c r="CW10" s="6"/>
+      <c r="CX10" s="6"/>
+      <c r="CY10" s="6"/>
+      <c r="CZ10" s="6"/>
+      <c r="DA10" s="6"/>
+      <c r="DB10" s="6"/>
+      <c r="DC10" s="6"/>
+      <c r="DD10" s="6"/>
+      <c r="DE10" s="6"/>
+      <c r="DF10" s="6"/>
+      <c r="DG10" s="6"/>
+      <c r="DH10" s="6"/>
+      <c r="DI10" s="6"/>
+      <c r="DJ10" s="6"/>
+      <c r="DK10" s="6"/>
+      <c r="DL10" s="6"/>
+      <c r="DM10" s="6"/>
+      <c r="DN10" s="6"/>
+      <c r="DO10" s="6"/>
+      <c r="DP10" s="6"/>
+      <c r="DQ10" s="6"/>
+      <c r="DR10" s="6"/>
+      <c r="DS10" s="6"/>
       <c r="DT10" s="6"/>
       <c r="DU10" s="6"/>
       <c r="DV10" s="6"/>
@@ -3743,28 +3718,28 @@
       <c r="FN10" s="6"/>
       <c r="FO10" s="6"/>
     </row>
-    <row r="11" spans="1:176" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:176" ht="90" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="E11" s="3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F11" s="3">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="G11" s="5">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
@@ -3858,78 +3833,94 @@
       <c r="CS11" s="6"/>
       <c r="CT11" s="6"/>
       <c r="CU11" s="6"/>
-      <c r="CV11" s="6"/>
-      <c r="CW11" s="6"/>
-      <c r="CX11" s="6"/>
-      <c r="CY11" s="6"/>
-      <c r="CZ11" s="6"/>
-      <c r="DA11" s="6"/>
-      <c r="DB11" s="6"/>
-      <c r="DC11" s="6"/>
-      <c r="DD11" s="6"/>
-      <c r="DE11" s="6"/>
-      <c r="DF11" s="6"/>
-      <c r="DG11" s="6"/>
-      <c r="DH11" s="6"/>
-      <c r="DI11" s="6"/>
-      <c r="DJ11" s="6"/>
-      <c r="DK11" s="6"/>
-      <c r="DL11" s="6"/>
-      <c r="DM11" s="6"/>
-      <c r="DN11" s="6"/>
-      <c r="DO11" s="6"/>
-      <c r="DP11" s="6"/>
-      <c r="DQ11" s="6"/>
-      <c r="DR11" s="6"/>
-      <c r="DS11" s="6"/>
-      <c r="DT11" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DU11" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DV11" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DW11" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DX11" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DY11" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="DZ11" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EA11" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EB11" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EC11" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="ED11" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EE11" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EF11" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EG11" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EH11" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EI11" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="CV11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CW11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CX11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CY11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="CZ11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DA11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DB11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DC11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DD11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DE11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DF11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DG11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DH11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DI11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DJ11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DK11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DL11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DM11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DN11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DO11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DP11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DQ11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DR11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DS11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DT11" s="6"/>
+      <c r="DU11" s="6"/>
+      <c r="DV11" s="6"/>
+      <c r="DW11" s="6"/>
+      <c r="DX11" s="6"/>
+      <c r="DY11" s="6"/>
+      <c r="DZ11" s="6"/>
+      <c r="EA11" s="6"/>
+      <c r="EB11" s="6"/>
+      <c r="EC11" s="6"/>
+      <c r="ED11" s="6"/>
+      <c r="EE11" s="6"/>
+      <c r="EF11" s="6"/>
+      <c r="EG11" s="6"/>
+      <c r="EH11" s="6"/>
+      <c r="EI11" s="6"/>
       <c r="EJ11" s="6"/>
       <c r="EK11" s="6"/>
       <c r="EL11" s="6"/>
@@ -3963,28 +3954,28 @@
       <c r="FN11" s="6"/>
       <c r="FO11" s="6"/>
     </row>
-    <row r="12" spans="1:176" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:176" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>203</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="E12" s="3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F12" s="3">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G12" s="5">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
@@ -4102,46 +4093,62 @@
       <c r="DQ12" s="6"/>
       <c r="DR12" s="6"/>
       <c r="DS12" s="6"/>
-      <c r="DT12" s="6"/>
-      <c r="DU12" s="6"/>
-      <c r="DV12" s="6"/>
-      <c r="DW12" s="6"/>
-      <c r="DX12" s="6"/>
-      <c r="DY12" s="6"/>
-      <c r="DZ12" s="6"/>
-      <c r="EA12" s="6"/>
-      <c r="EB12" s="6"/>
-      <c r="EC12" s="6"/>
-      <c r="ED12" s="6"/>
-      <c r="EE12" s="6"/>
-      <c r="EF12" s="6"/>
-      <c r="EG12" s="6"/>
-      <c r="EH12" s="6"/>
-      <c r="EI12" s="6"/>
-      <c r="EJ12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EK12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EL12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EM12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EN12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EO12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EP12" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EQ12" s="3" t="s">
-        <v>179</v>
-      </c>
+      <c r="DT12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DU12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DV12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DW12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DX12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DY12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="DZ12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EA12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EB12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EC12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="ED12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EE12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EF12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EG12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EH12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EI12" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EJ12" s="6"/>
+      <c r="EK12" s="6"/>
+      <c r="EL12" s="6"/>
+      <c r="EM12" s="6"/>
+      <c r="EN12" s="6"/>
+      <c r="EO12" s="6"/>
+      <c r="EP12" s="6"/>
+      <c r="EQ12" s="6"/>
       <c r="ER12" s="6"/>
       <c r="ES12" s="6"/>
       <c r="ET12" s="6"/>
@@ -4167,28 +4174,28 @@
       <c r="FN12" s="6"/>
       <c r="FO12" s="6"/>
     </row>
-    <row r="13" spans="1:176" ht="60" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:176" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="E13" s="3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F13" s="3">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="G13" s="5">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="H13" s="6"/>
       <c r="I13" s="6"/>
@@ -4322,90 +4329,294 @@
       <c r="EG13" s="6"/>
       <c r="EH13" s="6"/>
       <c r="EI13" s="6"/>
-      <c r="EJ13" s="6"/>
-      <c r="EK13" s="6"/>
-      <c r="EL13" s="6"/>
-      <c r="EM13" s="6"/>
-      <c r="EN13" s="6"/>
-      <c r="EO13" s="6"/>
-      <c r="EP13" s="6"/>
-      <c r="EQ13" s="6"/>
-      <c r="ER13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="ES13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="ET13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EU13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EV13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EW13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EX13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EY13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="EZ13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FA13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FB13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FC13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FD13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FE13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FF13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FG13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FH13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FI13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FJ13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FK13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FL13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FM13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FN13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="FO13" s="3" t="s">
+      <c r="EJ13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EK13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EL13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EM13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EN13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EO13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EP13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EQ13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="ER13" s="6"/>
+      <c r="ES13" s="6"/>
+      <c r="ET13" s="6"/>
+      <c r="EU13" s="6"/>
+      <c r="EV13" s="6"/>
+      <c r="EW13" s="6"/>
+      <c r="EX13" s="6"/>
+      <c r="EY13" s="6"/>
+      <c r="EZ13" s="6"/>
+      <c r="FA13" s="6"/>
+      <c r="FB13" s="6"/>
+      <c r="FC13" s="6"/>
+      <c r="FD13" s="6"/>
+      <c r="FE13" s="6"/>
+      <c r="FF13" s="6"/>
+      <c r="FG13" s="6"/>
+      <c r="FH13" s="6"/>
+      <c r="FI13" s="6"/>
+      <c r="FJ13" s="6"/>
+      <c r="FK13" s="6"/>
+      <c r="FL13" s="6"/>
+      <c r="FM13" s="6"/>
+      <c r="FN13" s="6"/>
+      <c r="FO13" s="6"/>
+    </row>
+    <row r="14" spans="1:176" ht="60" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="E14" s="3">
+        <v>5</v>
+      </c>
+      <c r="F14" s="3">
+        <v>24</v>
+      </c>
+      <c r="G14" s="5">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="6"/>
+      <c r="K14" s="6"/>
+      <c r="L14" s="6"/>
+      <c r="M14" s="6"/>
+      <c r="N14" s="6"/>
+      <c r="O14" s="6"/>
+      <c r="P14" s="6"/>
+      <c r="Q14" s="6"/>
+      <c r="R14" s="6"/>
+      <c r="S14" s="6"/>
+      <c r="T14" s="6"/>
+      <c r="U14" s="6"/>
+      <c r="V14" s="6"/>
+      <c r="W14" s="6"/>
+      <c r="X14" s="6"/>
+      <c r="Y14" s="6"/>
+      <c r="Z14" s="6"/>
+      <c r="AA14" s="6"/>
+      <c r="AB14" s="6"/>
+      <c r="AC14" s="6"/>
+      <c r="AD14" s="6"/>
+      <c r="AE14" s="6"/>
+      <c r="AF14" s="6"/>
+      <c r="AG14" s="6"/>
+      <c r="AH14" s="6"/>
+      <c r="AI14" s="6"/>
+      <c r="AJ14" s="6"/>
+      <c r="AK14" s="6"/>
+      <c r="AL14" s="6"/>
+      <c r="AM14" s="6"/>
+      <c r="AN14" s="6"/>
+      <c r="AO14" s="6"/>
+      <c r="AP14" s="6"/>
+      <c r="AQ14" s="6"/>
+      <c r="AR14" s="6"/>
+      <c r="AS14" s="6"/>
+      <c r="AT14" s="6"/>
+      <c r="AU14" s="6"/>
+      <c r="AV14" s="6"/>
+      <c r="AW14" s="6"/>
+      <c r="AX14" s="6"/>
+      <c r="AY14" s="6"/>
+      <c r="AZ14" s="6"/>
+      <c r="BA14" s="6"/>
+      <c r="BB14" s="6"/>
+      <c r="BC14" s="6"/>
+      <c r="BD14" s="6"/>
+      <c r="BE14" s="6"/>
+      <c r="BF14" s="6"/>
+      <c r="BG14" s="6"/>
+      <c r="BH14" s="6"/>
+      <c r="BI14" s="6"/>
+      <c r="BJ14" s="6"/>
+      <c r="BK14" s="6"/>
+      <c r="BL14" s="6"/>
+      <c r="BM14" s="6"/>
+      <c r="BN14" s="6"/>
+      <c r="BO14" s="6"/>
+      <c r="BP14" s="6"/>
+      <c r="BQ14" s="6"/>
+      <c r="BR14" s="6"/>
+      <c r="BS14" s="6"/>
+      <c r="BT14" s="6"/>
+      <c r="BU14" s="6"/>
+      <c r="BV14" s="6"/>
+      <c r="BW14" s="6"/>
+      <c r="BX14" s="6"/>
+      <c r="BY14" s="6"/>
+      <c r="BZ14" s="6"/>
+      <c r="CA14" s="6"/>
+      <c r="CB14" s="6"/>
+      <c r="CC14" s="6"/>
+      <c r="CD14" s="6"/>
+      <c r="CE14" s="6"/>
+      <c r="CF14" s="6"/>
+      <c r="CG14" s="6"/>
+      <c r="CH14" s="6"/>
+      <c r="CI14" s="6"/>
+      <c r="CJ14" s="6"/>
+      <c r="CK14" s="6"/>
+      <c r="CL14" s="6"/>
+      <c r="CM14" s="6"/>
+      <c r="CN14" s="6"/>
+      <c r="CO14" s="6"/>
+      <c r="CP14" s="6"/>
+      <c r="CQ14" s="6"/>
+      <c r="CR14" s="6"/>
+      <c r="CS14" s="6"/>
+      <c r="CT14" s="6"/>
+      <c r="CU14" s="6"/>
+      <c r="CV14" s="6"/>
+      <c r="CW14" s="6"/>
+      <c r="CX14" s="6"/>
+      <c r="CY14" s="6"/>
+      <c r="CZ14" s="6"/>
+      <c r="DA14" s="6"/>
+      <c r="DB14" s="6"/>
+      <c r="DC14" s="6"/>
+      <c r="DD14" s="6"/>
+      <c r="DE14" s="6"/>
+      <c r="DF14" s="6"/>
+      <c r="DG14" s="6"/>
+      <c r="DH14" s="6"/>
+      <c r="DI14" s="6"/>
+      <c r="DJ14" s="6"/>
+      <c r="DK14" s="6"/>
+      <c r="DL14" s="6"/>
+      <c r="DM14" s="6"/>
+      <c r="DN14" s="6"/>
+      <c r="DO14" s="6"/>
+      <c r="DP14" s="6"/>
+      <c r="DQ14" s="6"/>
+      <c r="DR14" s="6"/>
+      <c r="DS14" s="6"/>
+      <c r="DT14" s="6"/>
+      <c r="DU14" s="6"/>
+      <c r="DV14" s="6"/>
+      <c r="DW14" s="6"/>
+      <c r="DX14" s="6"/>
+      <c r="DY14" s="6"/>
+      <c r="DZ14" s="6"/>
+      <c r="EA14" s="6"/>
+      <c r="EB14" s="6"/>
+      <c r="EC14" s="6"/>
+      <c r="ED14" s="6"/>
+      <c r="EE14" s="6"/>
+      <c r="EF14" s="6"/>
+      <c r="EG14" s="6"/>
+      <c r="EH14" s="6"/>
+      <c r="EI14" s="6"/>
+      <c r="EJ14" s="6"/>
+      <c r="EK14" s="6"/>
+      <c r="EL14" s="6"/>
+      <c r="EM14" s="6"/>
+      <c r="EN14" s="6"/>
+      <c r="EO14" s="6"/>
+      <c r="EP14" s="6"/>
+      <c r="EQ14" s="6"/>
+      <c r="ER14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="ES14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="ET14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EU14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EV14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EW14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EX14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EY14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="EZ14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FA14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FB14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FC14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FD14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FE14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FF14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FG14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FH14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FI14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FJ14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FK14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FL14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FM14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FN14" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="FO14" s="3" t="s">
         <v>179</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="H5:FO5 AO6:FO6 H6:AM7 AN7:FO7">
+  <conditionalFormatting sqref="H5:FO5 AO6:FO6 H6:AM6 H7:FO8">
     <cfRule type="cellIs" dxfId="15" priority="13" operator="equal">
       <formula>"X"</formula>
     </cfRule>
@@ -4413,7 +4624,7 @@
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H8:FO8">
+  <conditionalFormatting sqref="H9:FO9">
     <cfRule type="cellIs" dxfId="13" priority="19" operator="equal">
       <formula>"X"</formula>
     </cfRule>
@@ -4421,7 +4632,7 @@
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H9:FO9">
+  <conditionalFormatting sqref="H10:FO10">
     <cfRule type="cellIs" dxfId="11" priority="21" operator="equal">
       <formula>"X"</formula>
     </cfRule>
@@ -4429,7 +4640,7 @@
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H10:FO10">
+  <conditionalFormatting sqref="H11:FO11">
     <cfRule type="cellIs" dxfId="9" priority="23" operator="equal">
       <formula>"X"</formula>
     </cfRule>
@@ -4437,7 +4648,7 @@
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H11:FO12">
+  <conditionalFormatting sqref="H12:FO13">
     <cfRule type="cellIs" dxfId="7" priority="25" operator="equal">
       <formula>"X"</formula>
     </cfRule>
@@ -4445,7 +4656,7 @@
       <formula>"x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H13:FO13">
+  <conditionalFormatting sqref="H14:FO14">
     <cfRule type="cellIs" dxfId="5" priority="29" operator="equal">
       <formula>"X"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Aggiornamento post sprint review
</commit_message>
<xml_diff>
--- a/7_Allegati/Sprint-planning.xlsx
+++ b/7_Allegati/Sprint-planning.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nqy271\BrutalBumperCars\bianchi-ciaponi-brutal-bumper-cars\7_Allegati\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Scuola\Anno_4\BrutalBumperCars(BBC)\7_Allegati\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D144A02-8816-4E75-BC35-6E0D98556A48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7657445-5135-4B2F-A1E7-14B051BE7C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gantt Orario Dettagliato" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="219">
   <si>
     <t>Sprint</t>
   </si>
@@ -699,13 +699,22 @@
   </si>
   <si>
     <t>Extra</t>
+  </si>
+  <si>
+    <t>• Animazioni menu presenti.
+• Dati salvati in DataBase SQLite.
+• Garage bozza presente.</t>
+  </si>
+  <si>
+    <t>• Il giocatore vede la mappa.
+• Gli elementi della mappa sono posizionati correttamente.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -726,6 +735,12 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -772,7 +787,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -790,6 +805,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -1291,7 +1309,7 @@
     <col min="1" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
     <col min="4" max="4" width="40" customWidth="1"/>
-    <col min="5" max="5" width="6" customWidth="1"/>
+    <col min="5" max="5" width="5.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="12" customWidth="1"/>
     <col min="8" max="176" width="2.42578125" customWidth="1"/>
   </cols>
@@ -2838,7 +2856,7 @@
       <c r="FN6" s="6"/>
       <c r="FO6" s="6"/>
     </row>
-    <row r="7" spans="1:176" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:176" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>182</v>
       </c>
@@ -2848,8 +2866,8 @@
       <c r="C7" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>191</v>
+      <c r="D7" s="7" t="s">
+        <v>218</v>
       </c>
       <c r="E7" s="3">
         <v>2</v>
@@ -3038,7 +3056,7 @@
       <c r="FN7" s="6"/>
       <c r="FO7" s="6"/>
     </row>
-    <row r="8" spans="1:176" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:176" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>182</v>
       </c>
@@ -3046,7 +3064,9 @@
       <c r="C8" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="D8" s="4"/>
+      <c r="D8" s="4" t="s">
+        <v>217</v>
+      </c>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
       <c r="G8" s="5">
@@ -4616,7 +4636,7 @@
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="H5:FO5 AO6:FO6 H6:AM6 H7:FO8">
+  <conditionalFormatting sqref="H5:FO5 H6:AM6 AO6:FO6 H7:FO8">
     <cfRule type="cellIs" dxfId="15" priority="13" operator="equal">
       <formula>"X"</formula>
     </cfRule>
@@ -4681,5 +4701,6 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
completamento visuale, aggiornamento gannt e diario
</commit_message>
<xml_diff>
--- a/7_Allegati/Sprint-planning.xlsx
+++ b/7_Allegati/Sprint-planning.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Scuola\Anno_4\BrutalBumperCars(BBC)\7_Allegati\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nqy271\BrutalBumperCars\bianchi-ciaponi-brutal-bumper-cars\7_Allegati\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7657445-5135-4B2F-A1E7-14B051BE7C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E02EC566-CB77-49E9-AFEA-3166C91E2CAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gantt Orario Dettagliato" sheetId="1" r:id="rId1"/>

</xml_diff>